<commit_message>
9961265 VMS day by day with charges and map links; branch workbook on the page's VMS model
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNRrrx1C9yJ5N627f7yfrr
</commit_message>
<xml_diff>
--- a/03_GC500_Delivery_Control/review_22Oct2026_baseplan6_schedule13/GC500_9961265_VMS_for_Branch_22Oct2026.xlsx
+++ b/03_GC500_Delivery_Control/review_22Oct2026_baseplan6_schedule13/GC500_9961265_VMS_for_Branch_22Oct2026.xlsx
@@ -1218,10 +1218,14 @@
           <t>2026-10-12</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>on our register (rego TF15JR) but no arrival day recorded</t>
+          <t>Andrew's word on the page: on site 2026-10-08</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1229,10 +1233,18 @@
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="L10" s="2" t="n"/>
-      <c r="M10" s="2" t="n"/>
-      <c r="N10" s="2" t="n"/>
-      <c r="O10" s="2" t="n"/>
+      <c r="L10" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="M10" s="3" t="n">
+        <v>804.17</v>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>965.01</v>
+      </c>
       <c r="P10" s="3" t="n">
         <v>1018.59</v>
       </c>
@@ -1253,79 +1265,95 @@
       </c>
       <c r="V10" s="2" t="inlineStr">
         <is>
-          <t>our record has no on-site day: start from the docket 2026-10-12 unless Andrew says otherwise</t>
+          <t>docket out 2026-10-12 differs from our day 2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" t="n">
         <v>13</v>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>VMS10</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>SUB-17093</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>120T</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>120T</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>V14221</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>not on our register</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Andrew's word on the page: on site 2026-10-08</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="L11" s="2" t="n"/>
-      <c r="M11" s="2" t="n"/>
-      <c r="N11" s="2" t="n"/>
-      <c r="O11" s="2" t="n"/>
-      <c r="P11" s="3" t="n">
+      <c r="L11" t="n">
+        <v>15</v>
+      </c>
+      <c r="M11" s="4" t="n">
+        <v>804.17</v>
+      </c>
+      <c r="N11" t="n">
+        <v>3</v>
+      </c>
+      <c r="O11" s="4" t="n">
+        <v>965.01</v>
+      </c>
+      <c r="P11" s="4" t="n">
         <v>1018.59</v>
       </c>
-      <c r="Q11" s="3" t="n">
+      <c r="Q11" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="R11" s="3" t="n">
-        <v>88.485</v>
-      </c>
-      <c r="S11" s="3" t="n">
-        <v>88.485</v>
-      </c>
-      <c r="T11" s="2" t="n">
-        <v>150</v>
-      </c>
-      <c r="U11" s="2" t="n">
-        <v>150</v>
-      </c>
-      <c r="V11" s="2" t="inlineStr">
-        <is>
-          <t>our register lacks fleet 120T - our fix, on Andrew's word; our record has no on-site day: start from the docket 2026-10-08 unless Andrew says otherwise</t>
-        </is>
-      </c>
+      <c r="R11" s="4" t="n">
+        <v>88.485</v>
+      </c>
+      <c r="S11" s="4" t="n">
+        <v>88.485</v>
+      </c>
+      <c r="T11" t="n">
+        <v>150</v>
+      </c>
+      <c r="U11" t="n">
+        <v>150</v>
+      </c>
+      <c r="V11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -2593,7 +2621,7 @@
       </c>
       <c r="V26" s="5" t="inlineStr">
         <is>
-          <t>Baseplan: a new board 1211356 for one day (20-21 Oct) with a $289.52 delivery. Our record: a board with rego ER9244 pinned at position 05a on 20 Oct 10:08 AEST (the plan's relocation of VMS05), still on site. Confirm 1211356 = ER9244; then the line stays on hire to demob (term 21 Oct is wrong) and the $289.52 is either a delivery or one of the $150 site shifts, not both</t>
+          <t>our register has 1211356 (rego ER9244) as the board at position 05a, pinned by Andrew 20 Oct 10:08 AEST, docket 26141143 the same morning, still on site: the line stays on hire to demob, so the 21 Oct term is wrong. The $289.52 delivery differs from the $150 a leg on line 41 - one rate or the other</t>
         </is>
       </c>
     </row>
@@ -2619,14 +2647,14 @@
       <c r="J28" s="7" t="inlineStr"/>
       <c r="K28" s="7" t="inlineStr"/>
       <c r="L28" s="7" t="n">
-        <v>390</v>
+        <v>420</v>
       </c>
       <c r="M28" s="8" t="n">
-        <v>20908.5</v>
+        <v>22516.84</v>
       </c>
       <c r="N28" s="7" t="inlineStr"/>
       <c r="O28" s="8" t="n">
-        <v>24982.96</v>
+        <v>26912.98</v>
       </c>
       <c r="P28" s="8" t="n">
         <v>33345.42</v>

</xml_diff>